<commit_message>
Update tiers (voice is Core+, not Spark) and expand skeleton spec
- Spark: buzzer only, no mic/speaker (AI tutor runs on laptop)
- Core: mic + speaker for on-robot voice AI
- Pro: mic array + HQ speaker for full conversational AI

Excel workbook now has 7 sheets:
- Global Variables, Section Boundaries, Joint Clearances (existing)
- Scaling Constraints (min/max for all parametric dimensions)
- Attachment Features (snap-fit clips, magnet recesses per section)
- Tier Upgrade Map (what stays/changes across Spark→Core→Pro)
- Magnet Spec (6×2mm N35 neodymium, recess dimensions, quantities)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/skeleton_exports/HawaBot_Spark_Skeleton_Parameters.xlsx
+++ b/pipeline/skeleton_exports/HawaBot_Spark_Skeleton_Parameters.xlsx
@@ -10,6 +10,10 @@
     <sheet name="Global Variables" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Section Boundaries" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Joint Clearances" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scaling Constraints" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Attachment Features" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tier Upgrade Map" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Magnet Spec" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2094,4 +2098,988 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Constraint Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>H_total (height)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Min: servos stacked vertically. Max: print bed height</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>BASE_W (width)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Min: Pi Pico W (51mm) + walls. Max: desk stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>BASE_D (depth)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Min: servo depth (13mm) + walls. Max: desk footprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>SHOULDER_X (spread)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Min: servo width + wall. Max: arm reach proportion</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TORSO_D (diameter)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Min: wire channel + wall. Max: proportion</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>T_wall (shell wall)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Min: FDM printability. Max: excessive weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>S (scale factor)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Derived from above constraints</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Magnet recess depth</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Min: magnet sits flush. Max: wall integrity</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Snap-fit hook overhang</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Min: holds. Max: hard to remove</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Attachment Type</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Dimensions &amp; Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>base_section</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Snap-fit clips</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>4× printed tabs</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Tab: 3mm wide × 2mm deep × 8mm tall. Hook overhang: 1.5mm. Located at corners of base top surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>base_section</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Magnet recess</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2× 6×2mm neodymium</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Recess: 6.2mm dia × 2.5mm deep. Top surface, for torso alignment. Centered at X=±15mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>torso_section</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Slide-on T-rails</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Printed as part of skeleton</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>T-profile: 2mm wide stem, 4mm wide cap, 1.5mm deep groove. 2× rails, full torso height on front and back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>torso_section</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Magnet recess (top)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2× 6×2mm neodymium</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Recess: 6.2mm dia × 2.5mm deep. Top surface for head connection. Centered at X=±8mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>torso_section</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Magnet recess (shoulders)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2× 6×2mm per side</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Recess: 6.2mm dia × 2.5mm deep. On shoulder mount face, for arm shell attachment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>left_arm_section</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Magnet recess</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2× 6×2mm neodymium</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Inner face, mates with torso shoulder magnets. Recess: 6.2mm dia × 2.5mm deep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>right_arm_section</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Magnet recess</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>2× 6×2mm neodymium</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Mirror of left arm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>head_section</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Magnet recess</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>3× 6×2mm neodymium</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>On mounting plate top surface. 120° spacing at R=8mm from center. Head shell pops on/off.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Spark ()</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Core ()</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Pro ()</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Head section</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>2× SG90 (pan+tilt)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>2× STS3215</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>2× XL330</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Torso section</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Column + shoulder stubs</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Column + full shoulder mounts</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Column + shoulder + waist roll</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Arm sections (each)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>1× MG90S (pitch only)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>3× STS3215 (pitch+roll+elbow)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>3× XL430/330 + wrist</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Base / legs</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Flat base, Pi Pico W</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Larger base, Pi 5</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Leg assembly replaces base, Pi 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>DOF total</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Buzzer only</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Mic + small speaker</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Mic array + 40mm speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Ultrasonic</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Ultrasonic + IMU</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Ultrasonic + IMU + camera + temp</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Teach-by-demo</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>No (no servo feedback)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Yes (STS3215 compliance)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Yes (Dynamixel Mode 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Keeps from prev tier</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Head shell, torso shell</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Head shell, torso shell</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>New parts needed</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Full kit</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Arm sections + base + servos</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Leg assembly + base + servos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Attachment type</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Snap-fit + magnets</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Same (compatible)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Same (compatible)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Magnet positions</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>10× 6×2mm</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>12× 6×2mm (+arm magnets)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>14× 6×2mm (+leg magnets)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Neodymium N35</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Standard hobby/craft grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Shape</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Disc</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Flat cylinder</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Diameter</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>6 mm</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Standard size, widely available</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2 mm</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Thin enough to embed in walls</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Recess diameter</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>6.2 mm</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>+0.2mm clearance for press fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Recess depth</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2.5 mm</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Magnet sits 0.5mm below surface (avoids snag)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Pull force (each)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>~0.5 kg</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Enough to hold shell, easy to pull off</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Cost per magnet</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>~$0.10</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Bulk pricing at 100+ qty</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Qty per Spark robot</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>10-12</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>~$1.00-1.20 total</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Polarity</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Mark one face</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Use sharpie dot on N pole, consistent orientation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Glue into recess</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Superglue (CA)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>One drop, press in, 30 sec cure</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>